<commit_message>
Added proper parameters for kalman model
</commit_message>
<xml_diff>
--- a/Data/Config_file.xlsx
+++ b/Data/Config_file.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Multi X Multi Y Optimization\Multi X Multi Y Optimization V2\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ankur.yadav\Desktop\Desktop Files\Soft_Sensor_and_What_If_Platform\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B1678F8-B108-402F-99B8-8F7C2C34ECF3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="user inputs" sheetId="1" r:id="rId1"/>
@@ -4272,7 +4271,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -4825,7 +4824,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -5003,7 +5002,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6A63DC9-6A36-42D7-A360-B87A5EA38E00}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -5141,7 +5140,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C840EB9-31CD-445F-875B-B69225FE1175}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -5401,7 +5400,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31B04680-28AE-4BED-AF57-53F49F6BB075}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I20"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -5841,7 +5840,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB249A9C-128C-47F2-A83B-0ABDBDE71708}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:EO9"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -9793,7 +9792,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{522A0632-3C09-466E-8133-C5BFEEA8B1C6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C519"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -15509,7 +15508,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAF2DDFA-3CEE-429D-BAFE-FF0BAF6E22FC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -15642,7 +15641,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F240B157-A43C-4900-871C-36D6279BDC26}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I19"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>

<commit_message>
Restructure the What-if Studio
</commit_message>
<xml_diff>
--- a/Data/Config_file.xlsx
+++ b/Data/Config_file.xlsx
@@ -9,13 +9,12 @@
   <sheets>
     <sheet name="PI_generalised_Name" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Model details" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="user inputs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Constraints" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Constraints" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="user inputs" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="display_column_order" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Model details_copy" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Section Order" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MV_DV_CV_taglist" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Target Section" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Section Order" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="MV_DV_CV_taglist" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Target Section" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -444,7 +443,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>GeneralizedDescription</t>
+          <t>Generalized Description</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -9765,7 +9764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9776,163 +9775,219 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>user input value</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Lower Limit</t>
+          <t>Max vlaue</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Upper Limit</t>
+          <t>UOM</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Remark</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Linked Parameter</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Action</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DMCTF_feed</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
+          <t>CGC_Turbine_HP_Steam_flow</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>230</v>
+      </c>
       <c r="C2" t="n">
-        <v>165000</v>
-      </c>
-      <c r="D2" t="n">
-        <v>205000</v>
+        <v>240</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>TPH</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>if user input is not there put None in the Value</t>
+          <t>If KT1310 stam flow &amp; KT1301 RPM &lt; user input value, then increase the speed to max</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>CGC_TURBINE_1_SPEED_(RPM)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>bump_linked_to_max</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Quench_tower_overhead_temp</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
+          <t>CGC_TURBINE_1_SPEED_(RPM)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4450</v>
+      </c>
       <c r="C3" t="n">
-        <v>32</v>
-      </c>
-      <c r="D3" t="n">
-        <v>50</v>
+        <v>4462</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>RPM</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CGC_TURBINE_1_SPEED_(RPM)</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="n">
-        <v>4250</v>
-      </c>
-      <c r="D4" t="n">
-        <v>4462</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>PRC_turbine_steam_flow</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>248</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TPH</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>If KT1601 stam flow &amp; KT1601 RPM &lt; user input value, then increase the speed to max</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PRC_turbine_RPM</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>bump_linked_to_max</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CGC_STAGE_1_SUCTION_PRESSURE</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
+          <t>PRC_turbine_RPM</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3700</v>
+      </c>
       <c r="C5" t="n">
-        <v>65</v>
-      </c>
-      <c r="D5" t="n">
-        <v>115</v>
+        <v>3724</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>RPM</t>
+        </is>
       </c>
       <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CGC_5TH_STG_DISCH_PRES</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="n">
-        <v>3700</v>
-      </c>
-      <c r="D6" t="n">
-        <v>3950</v>
-      </c>
-      <c r="E6" t="inlineStr"/>
+          <t>ERC_turbine_steam_flow</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>TPH</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>If KT1701 stam flow &amp; KT1701 RPM &lt; user input value, then increase the speed to max</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ERC_turbine_Speed</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>bump_linked_to_max</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PRC_turbine_RPM</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
+          <t>ERC_turbine_Speed</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>7600</v>
+      </c>
       <c r="C7" t="n">
-        <v>3550</v>
-      </c>
-      <c r="D7" t="n">
-        <v>3724</v>
+        <v>7613</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>RPM</t>
+        </is>
       </c>
       <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PRC_1ST_STAGE_Suction_PRESSURE</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="n">
-        <v>23.7</v>
-      </c>
-      <c r="D8" t="n">
-        <v>28.5</v>
-      </c>
-      <c r="E8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>ERC_turbine_Speed</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="n">
-        <v>7400</v>
-      </c>
-      <c r="D9" t="n">
-        <v>7613</v>
-      </c>
-      <c r="E9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>ERC_1ST_STAGE_Suction_PRESSURE</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="n">
-        <v>9</v>
-      </c>
-      <c r="D10" t="n">
-        <v>18</v>
-      </c>
-      <c r="E10" t="inlineStr"/>
+          <t>CGC_5TH_STG_DISCH_PRES</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3900</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>KPA</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>if discharge pressure &gt; user input value, then we can not push DMCTF feed further</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>abort_if_exceeds</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9945,7 +10000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9956,219 +10011,163 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>user input value</t>
+          <t>Value</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Max vlaue</t>
+          <t>Lower Limit</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>UOM</t>
+          <t>Upper Limit</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Remark</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Linked Parameter</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Action</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CGC_Turbine_HP_Steam_flow</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>230</v>
-      </c>
+          <t>DMCTF_feed</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>240</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>TPH</t>
-        </is>
+        <v>165000</v>
+      </c>
+      <c r="D2" t="n">
+        <v>205000</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>If KT1310 stam flow &amp; KT1301 RPM &lt; user input value, then increase the speed to max</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>CGC_TURBINE_1_SPEED_(RPM)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>bump_linked_to_max</t>
+          <t>if user input is not there put None in the Value</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CGC_TURBINE_1_SPEED_(RPM)</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>4450</v>
-      </c>
+          <t>Quench_tower_overhead_temp</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
-        <v>4462</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>RPM</t>
-        </is>
+        <v>32</v>
+      </c>
+      <c r="D3" t="n">
+        <v>50</v>
       </c>
       <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PRC_turbine_steam_flow</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>248</v>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>TPH</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>If KT1601 stam flow &amp; KT1601 RPM &lt; user input value, then increase the speed to max</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PRC_turbine_RPM</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>bump_linked_to_max</t>
-        </is>
-      </c>
+          <t>CGC_TURBINE_1_SPEED_(RPM)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="n">
+        <v>4250</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4462</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PRC_turbine_RPM</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>3700</v>
-      </c>
+          <t>CGC_STAGE_1_SUCTION_PRESSURE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" t="n">
-        <v>3724</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>RPM</t>
-        </is>
+        <v>65</v>
+      </c>
+      <c r="D5" t="n">
+        <v>115</v>
       </c>
       <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ERC_turbine_steam_flow</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>43.8</v>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>TPH</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>If KT1701 stam flow &amp; KT1701 RPM &lt; user input value, then increase the speed to max</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>ERC_turbine_Speed</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>bump_linked_to_max</t>
-        </is>
-      </c>
+          <t>CGC_5TH_STG_DISCH_PRES</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="n">
+        <v>3700</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3950</v>
+      </c>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ERC_turbine_Speed</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>7600</v>
-      </c>
+          <t>PRC_turbine_RPM</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="n">
-        <v>7613</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>RPM</t>
-        </is>
+        <v>3550</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3724</v>
       </c>
       <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CGC_5TH_STG_DISCH_PRES</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>3900</v>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>KPA</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>if discharge pressure &gt; user input value, then we can not push DMCTF feed further</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>abort_if_exceeds</t>
-        </is>
-      </c>
+          <t>PRC_1ST_STAGE_Suction_PRESSURE</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="D8" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="E8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ERC_turbine_Speed</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="n">
+        <v>7400</v>
+      </c>
+      <c r="D9" t="n">
+        <v>7613</v>
+      </c>
+      <c r="E9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ERC_1ST_STAGE_Suction_PRESSURE</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D10" t="n">
+        <v>18</v>
+      </c>
+      <c r="E10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10517,602 +10516,80 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Predicted parameter</t>
+          <t>Sr.no</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Input parameters</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 2</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 3</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 4</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 5</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 6</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 7</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 8</t>
+          <t>Section</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Quench tower overhead temp</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Top Reflux Temp</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Quench tower inlet temp</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Cooling water supply temp</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+          <t>Furnace</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>CGC STAGE 1 SUCTION PRESSURE</t>
-        </is>
+      <c r="A3" t="n">
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DMCTF feed</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Cooling water supply temp</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Quench tower overhead temp</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>KT1301 TURBINE SPEED (RPM)</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>KT1302 TURBINE SPEED (RPM)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Average interstage differential pressure</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+          <t>Quench</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Overall_COT</t>
-        </is>
+      <c r="A4" t="n">
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DMCTF feed</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CGC STAGE 1 SUCTION PRESSURE</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Furnace_conversion</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+          <t>CGC</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>K1302 5TH STG DISCH PRES</t>
-        </is>
+      <c r="A5" t="n">
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DMCTF feed</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+          <t>PRC</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>CGC_Power_KW</t>
-        </is>
+      <c r="A6" t="n">
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DMCTF feed</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CGC STAGE 1 SUCTION PRESSURE</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>K1302 5TH STG DISCH PRES</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>KT1301 TURBINE SPEED (RPM)</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Cooling water supply temp</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+          <t>ERC</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>CHG_GAS_FLOW_TO_DRYER</t>
-        </is>
+      <c r="A7" t="n">
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DMCTF feed</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>K1601 1ST STAGE Suction FLOW</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>DMCTF feed</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CGC STAGE 1 SUCTION PRESSURE</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>K1302 5TH STG DISCH PRES</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>KT1601 Turbine RPM</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>K1601 1ST STAGE Suction PRESSURE</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>DMCTF feed</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CGC STAGE 1 SUCTION PRESSURE</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>K1302 5TH STG DISCH PRES</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>KT1601 Turbine RPM</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>D1602 Overhead Flow</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>DMCTF feed</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Avg_MW</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>K1601 1ST STAGE Suction FLOW</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>K1601 1ST STAGE Suction PRESSURE</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>KT1601 Turbine RPM</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>K1601 1ST STAGE Suction TEMP</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>K1601_Total_estimated_power_MW</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>K1601 1ST STAGE Suction FLOW</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>K1601 1ST STAGE Suction PRESSURE</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>D1602 Overhead Flow</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>D1702 Overhead Flow</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>DMCTF feed</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>CGC STAGE 1 SUCTION PRESSURE</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>K1302 5TH STG DISCH PRES</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>KT1701 Turbine Speed</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>KT-1701 steam flow</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>KT-1701 steam flow</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>DMCTF feed</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>K1302 5TH STG DISCH PRES</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>K1701 1ST STAGE Suction FLOW</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>D1702 Overhead Flow</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>KT1701 Turbine Speed</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>ERC power</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>DMCTF feed</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>KT-1701 steam flow</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>K1701 1ST STAGE Suction FLOW</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>DMCTF feed</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>CGC STAGE 1 SUCTION PRESSURE</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>K1302 5TH STG DISCH PRES</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>KT1701 Turbine Speed</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>KT-1701 steam flow</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>K1701 1ST STAGE Suction PRESSURE</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>DMCTF feed</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>CGC STAGE 1 SUCTION PRESSURE</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>K1302 5TH STG DISCH PRES</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>KT1701 Turbine Speed</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>KT-1701 steam flow</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Cooling water supply temp</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>TOTAL ETHYLENE LOSS</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>DMCTF feed</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Demeth No2 feed flow</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Demeth tower pressure control OP</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>K1601 1ST STAGE Suction PRESSURE</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Demeth OH to condenser</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Demeth tower reflux temp</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Demeth feed separator OH valve opening</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Fresh ethane feed</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Ethylene product flow</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>DMCTF feed</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>CGC STAGE 1 SUCTION PRESSURE</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>K1302 5TH STG DISCH PRES</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>K1601 1ST STAGE Suction PRESSURE</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>D1702 Overhead Flow</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Fresh ethane feed</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
+          <t>Cold</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11125,82 +10602,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Sr.no</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Furnace</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Quench</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>CGC</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>PRC</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ERC</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11211,702 +10615,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>GeneralizedDescription</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>YN.ETH1.13P177</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>CGC_3RD_STG_DISCH_PRES</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CGC</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Dependent</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>YN.ETH1.13P185</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>CGC_5TH_STG_DISCH_PRES</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>CGC</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Dependent</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>YN.ETH1.18P267</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>PRC_turbine_Steam_pressure</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>PRC</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Independent</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>YN.ETH1.16PC237</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>PRC_3RD_STAGE_Discharge_PRESSURE</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>PRC</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Independent</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>YN.ETH1.16FC379</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PRC_turbine_Extraction_flow</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>PRC</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Independent</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>YN.ETH1.16P123</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>PRC_turbine_Condensate_chest_pressure</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>PRC</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Dependent</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>YN.ETH1.16P124</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>PRC_turbine_Extraction_chest_pressure</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>PRC</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Dependent</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>YN.ETH1.17PC241</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>ERC_1ST_STG_PRESS_CNTL</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>ERC</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>YN.ETH1.17PC902</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>ETHYL_REFRG_ACMLTR_Pressure_CNTL</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>ERC</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>YN.ETH1.16LC120</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>C2_Refrig_condenser_PR_LEVEL_CONTROL</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>ERC</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>YN.ETH1.14PC980</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Off_gas_exp_inlet_pressure</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Independent</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>YN.ETH1.14PC981</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Methane_expander_inlet_pressure</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Independent</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>YN.ETH1.14HC906OP</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Demeth_feed_separator_OH_valve_opening</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Independent</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>YN.ETH1.14FC299</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Deemthanizer_BTMS_flow_control</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Independent</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>YN.ETH1.14PD951</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>ERU-1_Mid_section_DP</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Dependent</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>YN.ETH1.14PD952</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>ERU-1_upper_section_DP</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Dependent</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>YN.ETH1.14PD950</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>ERU-2_differntial_pressure</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Dependent</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>YN.ETH1.14PC981OP</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Methane_exp_inlet_pressure_opening</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Dependent</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>YN.ETH1.14PC200</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>H2_Product_pressure_control</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Independent</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>YN.ETH1.14PC205</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Deemth_tower_pressure_control</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Independent</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>YN.ETH1.14FC298</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Demeth_tower_reflux_flow</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Independent</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>YN.ETH1.14PCT428</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Demeth_tower_pressure_comp_temp_CNTL</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Independent</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>YN.ETH1.14PD201</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>DeltaP_Demeth_coldbox</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Dependent</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>YN.ETH1.14PC205OP</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Demeth_tower_pressure_control_OP</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Dependent</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>YN.ETH1.14LC085</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Demeth_Reflux_drum_level</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Dependent</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>YN.ETH1.14T433</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Demeth_Overhead_temp</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Independent</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>YN.ETH1.14AT091C</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Demeth_BTMS_Methane_ppm</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Dependent</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>YN.ETH1.14PD202</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Demeth_tower_deltaP</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Dependent</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>YN.ETH1.17LC137OP</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Demeth_Overhead_condenser_LVL_control_OP</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Dependent</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>YN.ETH1.16FC335</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Demeth_reboiler_Propylene_flow</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Dependent</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -11920,7 +10628,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>PRC</t>
         </is>
       </c>
     </row>

</xml_diff>